<commit_message>
add api/main.py, schema.sql修改, line程式碼調整
</commit_message>
<xml_diff>
--- a/document/資料庫、資料處理/假資料_範例.xlsx
+++ b/document/資料庫、資料處理/假資料_範例.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026/06/15 07:17:05</t>
+          <t>2026/06/18 11:46:04</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -600,12 +600,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026/11/08</t>
+          <t>2026/11/11</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026/11/16</t>
+          <t>2026/11/19</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/08~2026/11/16 (測試)</t>
+          <t>服務期間:2026/11/11~2026/11/19 (測試)</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026/06/03 23:04:45</t>
+          <t>2026/06/07 03:33:44</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -711,12 +711,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026/11/02</t>
+          <t>2026/11/05</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026/11/05</t>
+          <t>2026/11/08</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/02~2026/11/05 (測試)</t>
+          <t>服務期間:2026/11/05~2026/11/08 (測試)</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026/06/20 05:41:49</t>
+          <t>2026/06/23 10:10:48</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -826,12 +826,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026/10/22</t>
+          <t>2026/10/25</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026/10/28</t>
+          <t>2026/10/31</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/22~2026/10/28 (測試)</t>
+          <t>服務期間:2026/10/25~2026/10/31 (測試)</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026/07/05 19:00:16</t>
+          <t>2026/07/08 23:29:15</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -937,12 +937,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026/08/15</t>
+          <t>2026/08/18</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026/08/19</t>
+          <t>2026/08/22</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/15~2026/08/19 (測試)</t>
+          <t>服務期間:2026/08/18~2026/08/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026/06/24 19:41:49</t>
+          <t>2026/06/28 00:10:48</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026/10/27</t>
+          <t>2026/10/30</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026/10/31</t>
+          <t>2026/11/03</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/27~2026/10/31 (測試)</t>
+          <t>服務期間:2026/10/30~2026/11/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026/06/07 18:44:53</t>
+          <t>2026/06/10 23:13:52</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026/11/04</t>
+          <t>2026/11/07</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026/11/13</t>
+          <t>2026/11/16</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/04~2026/11/13 (測試)</t>
+          <t>服務期間:2026/11/07~2026/11/16 (測試)</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026/06/04 07:50:49</t>
+          <t>2026/06/07 12:19:48</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026/11/22</t>
+          <t>2026/11/25</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026/12/01</t>
+          <t>2026/12/04</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/22~2026/12/01 (測試)</t>
+          <t>服務期間:2026/11/25~2026/12/04 (測試)</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026/07/04 19:17:08</t>
+          <t>2026/07/07 23:46:07</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1385,12 +1385,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026/10/19</t>
+          <t>2026/10/22</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026/10/28</t>
+          <t>2026/10/31</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/19~2026/10/28 (測試)</t>
+          <t>服務期間:2026/10/22~2026/10/31 (測試)</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026/06/03 17:56:03</t>
+          <t>2026/06/06 22:25:02</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1496,12 +1496,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026/08/30</t>
+          <t>2026/09/02</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026/09/03</t>
+          <t>2026/09/06</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/30~2026/09/03 (測試)</t>
+          <t>服務期間:2026/09/02~2026/09/06 (測試)</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026/07/14 12:53:44</t>
+          <t>2026/07/17 17:22:43</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026/11/21</t>
+          <t>2026/11/24</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026/11/29</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/21~2026/11/29 (測試)</t>
+          <t>服務期間:2026/11/24~2026/12/02 (測試)</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026/07/01 17:11:15</t>
+          <t>2026/07/04 21:40:14</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1718,12 +1718,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2026/11/26</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/23~2026/11/30 (測試)</t>
+          <t>服務期間:2026/11/26~2026/12/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026/06/01 19:42:33</t>
+          <t>2026/06/05 00:11:32</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1829,12 +1829,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026/09/20</t>
+          <t>2026/09/23</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/10~2026/09/20 (測試)</t>
+          <t>服務期間:2026/09/13~2026/09/23 (測試)</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026/06/07 17:20:42</t>
+          <t>2026/06/10 21:49:41</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026/11/11</t>
+          <t>2026/11/14</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026/11/16</t>
+          <t>2026/11/19</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/11~2026/11/16 (測試)</t>
+          <t>服務期間:2026/11/14~2026/11/19 (測試)</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026/05/31 02:20:38</t>
+          <t>2026/06/03 06:49:37</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026/08/29</t>
+          <t>2026/09/01</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026/09/05</t>
+          <t>2026/09/08</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/29~2026/09/05 (測試)</t>
+          <t>服務期間:2026/09/01~2026/09/08 (測試)</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026/05/30 21:41:47</t>
+          <t>2026/06/03 02:10:46</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2166,12 +2166,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026/11/10</t>
+          <t>2026/11/13</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026/11/19</t>
+          <t>2026/11/22</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/10~2026/11/19 (測試)</t>
+          <t>服務期間:2026/11/13~2026/11/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026/06/04 10:33:25</t>
+          <t>2026/06/07 15:02:24</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2277,12 +2277,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026/11/16</t>
+          <t>2026/11/19</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026/11/19</t>
+          <t>2026/11/22</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/16~2026/11/19 (測試)</t>
+          <t>服務期間:2026/11/19~2026/11/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026/06/23 16:24:49</t>
+          <t>2026/06/26 20:53:48</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2392,12 +2392,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026/09/02</t>
+          <t>2026/09/05</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/02~2026/09/10 (測試)</t>
+          <t>服務期間:2026/09/05~2026/09/13 (測試)</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026/07/11 07:59:40</t>
+          <t>2026/07/14 12:28:39</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026/11/28</t>
+          <t>2026/12/01</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026/12/04</t>
+          <t>2026/12/07</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/28~2026/12/04 (測試)</t>
+          <t>服務期間:2026/12/01~2026/12/07 (測試)</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026/06/25 21:07:42</t>
+          <t>2026/06/29 01:36:41</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2618,12 +2618,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026/10/06</t>
+          <t>2026/10/09</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026/10/12</t>
+          <t>2026/10/15</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/06~2026/10/12 (測試)</t>
+          <t>服務期間:2026/10/09~2026/10/15 (測試)</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026/07/03 12:42:34</t>
+          <t>2026/07/06 17:11:33</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2729,12 +2729,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026/10/24</t>
+          <t>2026/10/27</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026/10/31</t>
+          <t>2026/11/03</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/24~2026/10/31 (測試)</t>
+          <t>服務期間:2026/10/27~2026/11/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026/05/18 15:42:30</t>
+          <t>2026/05/21 20:11:29</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2027/01/07</t>
+          <t>2027/01/10</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2027/01/13</t>
+          <t>2027/01/16</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>服務期間:2027/01/07~2027/01/13 (測試)</t>
+          <t>服務期間:2027/01/10~2027/01/16 (測試)</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026/05/22 03:51:56</t>
+          <t>2026/05/25 08:20:55</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2955,12 +2955,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026/10/06</t>
+          <t>2026/10/09</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/06~2026/10/09 (測試)</t>
+          <t>服務期間:2026/10/09~2026/10/12 (測試)</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026/06/27 16:14:57</t>
+          <t>2026/06/30 20:43:56</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026/09/02</t>
+          <t>2026/09/05</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/02~2026/09/10 (測試)</t>
+          <t>服務期間:2026/09/05~2026/09/13 (測試)</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026/07/01 05:17:09</t>
+          <t>2026/07/04 09:46:08</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3177,12 +3177,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026/12/23</t>
+          <t>2026/12/26</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/23~2026/12/29 (測試)</t>
+          <t>服務期間:2026/12/26~2027/01/01 (測試)</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026/06/18 03:29:32</t>
+          <t>2026/06/21 07:58:31</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3288,12 +3288,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026/10/23</t>
+          <t>2026/10/26</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026/10/31</t>
+          <t>2026/11/03</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/23~2026/10/31 (測試)</t>
+          <t>服務期間:2026/10/26~2026/11/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026/07/02 18:04:07</t>
+          <t>2026/07/05 22:33:06</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3399,12 +3399,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026/11/08</t>
+          <t>2026/11/11</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026/11/18</t>
+          <t>2026/11/21</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/08~2026/11/18 (測試)</t>
+          <t>服務期間:2026/11/11~2026/11/21 (測試)</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3469,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026/07/12 05:20:54</t>
+          <t>2026/07/15 09:49:53</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3514,12 +3514,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026/12/19</t>
+          <t>2026/12/22</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/19~2026/12/29 (測試)</t>
+          <t>服務期間:2026/12/22~2027/01/01 (測試)</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026/06/02 23:50:03</t>
+          <t>2026/06/06 04:19:02</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/27</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/18~2026/08/24 (測試)</t>
+          <t>服務期間:2026/08/21~2026/08/27 (測試)</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026/07/09 02:48:57</t>
+          <t>2026/07/12 07:17:56</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3740,12 +3740,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026/10/15</t>
+          <t>2026/10/18</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026/10/25</t>
+          <t>2026/10/28</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/15~2026/10/25 (測試)</t>
+          <t>服務期間:2026/10/18~2026/10/28 (測試)</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026/05/30 05:07:50</t>
+          <t>2026/06/02 09:36:49</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3851,12 +3851,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026/12/15</t>
+          <t>2026/12/18</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026/12/21</t>
+          <t>2026/12/24</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/15~2026/12/21 (測試)</t>
+          <t>服務期間:2026/12/18~2026/12/24 (測試)</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026/07/02 18:25:54</t>
+          <t>2026/07/05 22:54:53</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3962,12 +3962,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026/11/25</t>
+          <t>2026/11/28</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026/12/04</t>
+          <t>2026/12/07</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/25~2026/12/04 (測試)</t>
+          <t>服務期間:2026/11/28~2026/12/07 (測試)</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026/07/01 04:18:24</t>
+          <t>2026/07/04 08:47:23</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4073,12 +4073,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026/11/25</t>
+          <t>2026/11/28</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026/12/02</t>
+          <t>2026/12/05</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/25~2026/12/02 (測試)</t>
+          <t>服務期間:2026/11/28~2026/12/05 (測試)</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026/06/17 02:22:18</t>
+          <t>2026/06/20 06:51:17</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4184,12 +4184,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026/12/27</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/27~2026/12/31 (測試)</t>
+          <t>服務期間:2026/12/30~2027/01/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026/05/19 12:00:38</t>
+          <t>2026/05/22 16:29:37</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026/09/07</t>
+          <t>2026/09/10</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026/09/12</t>
+          <t>2026/09/15</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/07~2026/09/12 (測試)</t>
+          <t>服務期間:2026/09/10~2026/09/15 (測試)</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026/05/20 04:02:51</t>
+          <t>2026/05/23 08:31:50</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4406,12 +4406,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026/10/05</t>
+          <t>2026/10/08</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/05~2026/10/09 (測試)</t>
+          <t>服務期間:2026/10/08~2026/10/12 (測試)</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026/06/25 22:27:49</t>
+          <t>2026/06/29 02:56:49</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4517,12 +4517,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026/11/08</t>
+          <t>2026/11/11</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026/11/15</t>
+          <t>2026/11/18</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/08~2026/11/15 (測試)</t>
+          <t>服務期間:2026/11/11~2026/11/18 (測試)</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026/06/03 19:55:54</t>
+          <t>2026/06/07 00:24:54</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4628,12 +4628,12 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026/10/22</t>
+          <t>2026/10/25</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026/10/26</t>
+          <t>2026/10/29</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/22~2026/10/26 (測試)</t>
+          <t>服務期間:2026/10/25~2026/10/29 (測試)</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026/05/27 13:18:06</t>
+          <t>2026/05/30 17:47:06</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4739,12 +4739,12 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026/10/17</t>
+          <t>2026/10/20</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/09~2026/10/17 (測試)</t>
+          <t>服務期間:2026/10/12~2026/10/20 (測試)</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026/06/06 13:40:45</t>
+          <t>2026/06/09 18:09:45</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4850,12 +4850,12 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026/10/30</t>
+          <t>2026/11/02</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026/11/04</t>
+          <t>2026/11/07</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/30~2026/11/04 (測試)</t>
+          <t>服務期間:2026/11/02~2026/11/07 (測試)</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026/07/04 22:57:15</t>
+          <t>2026/07/08 03:26:15</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026/09/13</t>
+          <t>2026/09/16</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026/09/20</t>
+          <t>2026/09/23</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/13~2026/09/20 (測試)</t>
+          <t>服務期間:2026/09/16~2026/09/23 (測試)</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026/05/18 12:14:34</t>
+          <t>2026/05/21 16:43:34</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5072,12 +5072,12 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026/09/04</t>
+          <t>2026/09/07</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026/09/08</t>
+          <t>2026/09/11</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/04~2026/09/08 (測試)</t>
+          <t>服務期間:2026/09/07~2026/09/11 (測試)</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026/07/02 18:00:39</t>
+          <t>2026/07/05 22:29:39</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5183,12 +5183,12 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026/09/16</t>
+          <t>2026/09/19</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/10~2026/09/16 (測試)</t>
+          <t>服務期間:2026/09/13~2026/09/19 (測試)</t>
         </is>
       </c>
     </row>
@@ -5249,7 +5249,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026/06/03 08:39:08</t>
+          <t>2026/06/06 13:08:08</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5294,12 +5294,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026/09/29</t>
+          <t>2026/10/02</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/29~2026/10/09 (測試)</t>
+          <t>服務期間:2026/10/02~2026/10/12 (測試)</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026/06/17 20:45:08</t>
+          <t>2026/06/21 01:14:08</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5409,12 +5409,12 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026/08/30</t>
+          <t>2026/09/02</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026/09/05</t>
+          <t>2026/09/08</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/30~2026/09/05 (測試)</t>
+          <t>服務期間:2026/09/02~2026/09/08 (測試)</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026/06/26 09:10:45</t>
+          <t>2026/06/29 13:39:45</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5520,12 +5520,12 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026/08/25</t>
+          <t>2026/08/28</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/18~2026/08/25 (測試)</t>
+          <t>服務期間:2026/08/21~2026/08/28 (測試)</t>
         </is>
       </c>
     </row>
@@ -5586,7 +5586,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026/06/26 16:01:29</t>
+          <t>2026/06/29 20:30:29</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5631,12 +5631,12 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026/12/03</t>
+          <t>2026/12/06</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026/12/08</t>
+          <t>2026/12/11</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/03~2026/12/08 (測試)</t>
+          <t>服務期間:2026/12/06~2026/12/11 (測試)</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026/05/25 05:11:52</t>
+          <t>2026/05/28 09:40:52</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5742,12 +5742,12 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2027/01/10</t>
+          <t>2027/01/13</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2027/01/19</t>
+          <t>2027/01/22</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5789,7 +5789,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>服務期間:2027/01/10~2027/01/19 (測試)</t>
+          <t>服務期間:2027/01/13~2027/01/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026/05/29 16:53:54</t>
+          <t>2026/06/01 21:22:54</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5853,12 +5853,12 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026/10/14</t>
+          <t>2026/10/17</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026/10/23</t>
+          <t>2026/10/26</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/14~2026/10/23 (測試)</t>
+          <t>服務期間:2026/10/17~2026/10/26 (測試)</t>
         </is>
       </c>
     </row>
@@ -5923,7 +5923,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026/06/04 21:10:58</t>
+          <t>2026/06/08 01:39:58</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5968,12 +5968,12 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026/08/16</t>
+          <t>2026/08/19</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026/08/26</t>
+          <t>2026/08/29</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/16~2026/08/26 (測試)</t>
+          <t>服務期間:2026/08/19~2026/08/29 (測試)</t>
         </is>
       </c>
     </row>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026/06/17 06:48:49</t>
+          <t>2026/06/20 11:17:49</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -6083,12 +6083,12 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026/10/22</t>
+          <t>2026/10/25</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026/10/27</t>
+          <t>2026/10/30</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/22~2026/10/27 (測試)</t>
+          <t>服務期間:2026/10/25~2026/10/30 (測試)</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026/05/19 15:35:47</t>
+          <t>2026/05/22 20:04:47</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026/06/20 10:24:02</t>
+          <t>2026/06/23 14:53:02</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026/06/29 14:36:34</t>
+          <t>2026/07/02 19:05:34</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026/06/06 16:36:08</t>
+          <t>2026/06/09 21:05:08</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -7304,7 +7304,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026/05/16 03:56:18</t>
+          <t>2026/05/19 08:25:18</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026/05/23 13:32:37</t>
+          <t>2026/05/26 18:01:37</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026/05/19 00:32:03</t>
+          <t>2026/05/22 05:01:03</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026/05/26 09:37:08</t>
+          <t>2026/05/29 14:06:08</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -8172,7 +8172,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026/06/18 18:50:29</t>
+          <t>2026/06/21 23:19:29</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026/06/12 04:43:00</t>
+          <t>2026/06/15 09:12:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026/06/21 14:01:34</t>
+          <t>2026/06/24 18:30:34</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026/06/20 20:27:40</t>
+          <t>2026/06/24 00:56:40</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026/05/29 11:28:31</t>
+          <t>2026/06/01 15:57:31</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026/05/15 11:13:18</t>
+          <t>2026/05/18 15:42:18</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026/05/16 12:08:14</t>
+          <t>2026/05/19 16:37:14</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026/06/20 15:47:45</t>
+          <t>2026/06/23 20:16:45</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026/06/28 03:24:22</t>
+          <t>2026/07/01 07:53:22</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -10157,7 +10157,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026/06/15 06:42:21</t>
+          <t>2026/06/18 11:11:21</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026/05/17 20:29:55</t>
+          <t>2026/05/21 00:58:55</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -10599,7 +10599,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026/06/13 07:59:22</t>
+          <t>2026/06/16 12:28:22</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026/06/19 12:52:40</t>
+          <t>2026/06/22 17:21:40</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026/05/23 06:04:12</t>
+          <t>2026/05/26 10:33:12</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -11282,7 +11282,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026/07/08 04:19:46</t>
+          <t>2026/07/11 08:48:46</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -11495,7 +11495,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026/07/03 07:26:50</t>
+          <t>2026/07/06 11:55:50</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026/05/28 12:24:00</t>
+          <t>2026/05/31 16:53:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026/06/14 08:12:22</t>
+          <t>2026/06/17 12:41:22</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026/05/24 10:46:53</t>
+          <t>2026/05/27 15:15:53</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -12391,7 +12391,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026/06/10 06:27:54</t>
+          <t>2026/06/13 10:56:54</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -12620,7 +12620,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026/05/18 00:25:35</t>
+          <t>2026/05/21 04:54:35</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -12837,7 +12837,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026/06/19 08:39:46</t>
+          <t>2026/06/22 13:08:46</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026/07/01 00:39:29</t>
+          <t>2026/07/04 05:08:29</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026/06/29 13:12:13</t>
+          <t>2026/07/02 17:41:13</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026/05/18 00:53:02</t>
+          <t>2026/05/21 05:22:02</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026/07/01 21:19:08</t>
+          <t>2026/07/05 01:48:08</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -13946,7 +13946,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026/05/23 03:11:48</t>
+          <t>2026/05/26 07:40:48</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -14159,7 +14159,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026/06/15 03:09:33</t>
+          <t>2026/06/18 07:38:33</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026/07/12 09:06:12</t>
+          <t>2026/07/15 13:35:12</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -14593,7 +14593,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026/05/15 14:48:53</t>
+          <t>2026/05/18 19:17:53</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -14818,7 +14818,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026/05/24 02:36:03</t>
+          <t>2026/05/27 07:05:03</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -15047,7 +15047,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026/06/06 11:18:19</t>
+          <t>2026/06/09 15:47:19</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -15268,7 +15268,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026/07/07 07:17:01</t>
+          <t>2026/07/10 11:46:01</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026/07/05 03:54:24</t>
+          <t>2026/07/08 08:23:24</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026/07/07 00:51:56</t>
+          <t>2026/07/10 05:20:56</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -15939,7 +15939,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026/06/26 20:54:42</t>
+          <t>2026/06/30 01:23:42</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -16152,7 +16152,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026/05/18 01:40:47</t>
+          <t>2026/05/21 06:09:47</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -16369,7 +16369,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026/06/23 18:58:40</t>
+          <t>2026/06/26 23:27:40</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -16590,7 +16590,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026/07/08 14:56:16</t>
+          <t>2026/07/11 19:25:16</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026/07/04 07:51:15</t>
+          <t>2026/07/07 12:20:15</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -17000,7 +17000,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026/05/17 20:06:39</t>
+          <t>2026/05/21 00:35:39</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -17217,7 +17217,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026/07/03 08:08:29</t>
+          <t>2026/07/06 12:37:29</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -17920,7 +17920,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>06-15 07:17</t>
+          <t>06-18 11:46</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -18224,7 +18224,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>06-03 23:04</t>
+          <t>06-07 03:33</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -18520,7 +18520,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>06-20 05:41</t>
+          <t>06-23 10:10</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -18820,7 +18820,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>07-05 19:00</t>
+          <t>07-08 23:29</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -19120,7 +19120,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>06-24 19:41</t>
+          <t>06-28 00:10</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -19416,7 +19416,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>06-07 18:44</t>
+          <t>06-10 23:13</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -19736,7 +19736,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>06-04 07:50</t>
+          <t>06-07 12:19</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -20036,7 +20036,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>07-04 19:17</t>
+          <t>07-07 23:46</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -20344,7 +20344,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>06-03 17:56</t>
+          <t>06-06 22:25</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -20644,7 +20644,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>07-14 12:53</t>
+          <t>07-17 17:22</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -20956,7 +20956,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>07-01 17:11</t>
+          <t>07-04 21:40</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -21252,7 +21252,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>06-01 19:42</t>
+          <t>06-05 00:11</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -21552,7 +21552,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>06-07 17:20</t>
+          <t>06-10 21:49</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -21852,7 +21852,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>05-31 02:20</t>
+          <t>06-03 06:49</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -22168,7 +22168,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>05-30 21:41</t>
+          <t>06-03 02:10</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -22496,7 +22496,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>06-04 10:33</t>
+          <t>06-07 15:02</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -22788,7 +22788,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>06-23 16:24</t>
+          <t>06-26 20:53</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -23072,7 +23072,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>07-11 07:59</t>
+          <t>07-14 12:28</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -23380,7 +23380,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>06-25 21:07</t>
+          <t>06-29 01:36</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -23680,7 +23680,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>07-03 12:42</t>
+          <t>07-06 17:11</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -23988,7 +23988,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>05-18 15:42</t>
+          <t>05-21 20:11</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -24268,7 +24268,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>05-22 03:51</t>
+          <t>05-25 08:20</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -24572,7 +24572,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>06-27 16:14</t>
+          <t>06-30 20:43</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -24884,7 +24884,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>07-01 05:17</t>
+          <t>07-04 09:46</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>06-18 03:29</t>
+          <t>06-21 07:58</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -25500,7 +25500,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>07-02 18:04</t>
+          <t>07-05 22:33</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -25800,7 +25800,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>07-12 05:20</t>
+          <t>07-15 09:49</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -26100,7 +26100,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>06-02 23:50</t>
+          <t>06-06 04:19</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -26408,7 +26408,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>07-09 02:48</t>
+          <t>07-12 07:17</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -26720,7 +26720,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>05-30 05:07</t>
+          <t>06-02 09:36</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -27008,7 +27008,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>07-02 18:25</t>
+          <t>07-05 22:54</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -27304,7 +27304,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>07-01 04:18</t>
+          <t>07-04 08:47</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -27604,7 +27604,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>06-17 02:22</t>
+          <t>06-20 06:51</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -27892,7 +27892,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>05-19 12:00</t>
+          <t>05-22 16:29</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -28204,7 +28204,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>05-20 04:02</t>
+          <t>05-23 08:31</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -28516,7 +28516,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>06-25 22:27</t>
+          <t>06-29 02:56</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -28808,7 +28808,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>06-03 19:55</t>
+          <t>06-07 00:24</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -29092,7 +29092,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>05-27 13:18</t>
+          <t>05-30 17:47</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -29404,7 +29404,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>06-06 13:40</t>
+          <t>06-09 18:09</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -29708,7 +29708,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>07-04 22:57</t>
+          <t>07-08 03:26</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -30000,7 +30000,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>05-18 12:14</t>
+          <t>05-21 16:43</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -30304,7 +30304,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>07-02 18:00</t>
+          <t>07-05 22:29</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -30600,7 +30600,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>06-03 08:39</t>
+          <t>06-06 13:08</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -30920,7 +30920,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>06-17 20:45</t>
+          <t>06-21 01:14</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -31228,7 +31228,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>06-26 09:10</t>
+          <t>06-29 13:39</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -31536,7 +31536,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>06-26 16:01</t>
+          <t>06-29 20:30</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -31844,7 +31844,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>05-25 05:11</t>
+          <t>05-28 09:40</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -32132,7 +32132,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>05-29 16:53</t>
+          <t>06-01 21:22</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -32428,7 +32428,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>06-04 21:10</t>
+          <t>06-08 01:39</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -32728,7 +32728,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>06-17 06:48</t>
+          <t>06-20 11:17</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">

</xml_diff>

<commit_message>
Line bot wen (#28)
* 修正合併後LINE Bot無法啟動bug

* 修正bug

* 新增line api接口

* 修正line bug

* schema新增table,start.bat新增fastapi&ngrok啟動,delete scratch/一次性腳本

* add api/main.py, schema.sql修改, line程式碼調整

* .json檔重購

* 新增webhook安全性驗證程序及去重,新增伺服器監控功能

* feat: strengthen LINE webhook and confirmation workflows

* caregiver改為staff統一名稱,移除驗證碼改為後台工作人員直接確認
</commit_message>
<xml_diff>
--- a/document/資料庫、資料處理/假資料_範例.xlsx
+++ b/document/資料庫、資料處理/假資料_範例.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026/06/15 07:17:05</t>
+          <t>2026/06/18 11:46:04</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -600,12 +600,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026/11/08</t>
+          <t>2026/11/11</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026/11/16</t>
+          <t>2026/11/19</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/08~2026/11/16 (測試)</t>
+          <t>服務期間:2026/11/11~2026/11/19 (測試)</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026/06/03 23:04:45</t>
+          <t>2026/06/07 03:33:44</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -711,12 +711,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026/11/02</t>
+          <t>2026/11/05</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026/11/05</t>
+          <t>2026/11/08</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/02~2026/11/05 (測試)</t>
+          <t>服務期間:2026/11/05~2026/11/08 (測試)</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026/06/20 05:41:49</t>
+          <t>2026/06/23 10:10:48</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -826,12 +826,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026/10/22</t>
+          <t>2026/10/25</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026/10/28</t>
+          <t>2026/10/31</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/22~2026/10/28 (測試)</t>
+          <t>服務期間:2026/10/25~2026/10/31 (測試)</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026/07/05 19:00:16</t>
+          <t>2026/07/08 23:29:15</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -937,12 +937,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026/08/15</t>
+          <t>2026/08/18</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026/08/19</t>
+          <t>2026/08/22</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/15~2026/08/19 (測試)</t>
+          <t>服務期間:2026/08/18~2026/08/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026/06/24 19:41:49</t>
+          <t>2026/06/28 00:10:48</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026/10/27</t>
+          <t>2026/10/30</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026/10/31</t>
+          <t>2026/11/03</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/27~2026/10/31 (測試)</t>
+          <t>服務期間:2026/10/30~2026/11/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026/06/07 18:44:53</t>
+          <t>2026/06/10 23:13:52</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026/11/04</t>
+          <t>2026/11/07</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026/11/13</t>
+          <t>2026/11/16</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/04~2026/11/13 (測試)</t>
+          <t>服務期間:2026/11/07~2026/11/16 (測試)</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026/06/04 07:50:49</t>
+          <t>2026/06/07 12:19:48</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026/11/22</t>
+          <t>2026/11/25</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026/12/01</t>
+          <t>2026/12/04</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/22~2026/12/01 (測試)</t>
+          <t>服務期間:2026/11/25~2026/12/04 (測試)</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026/07/04 19:17:08</t>
+          <t>2026/07/07 23:46:07</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1385,12 +1385,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026/10/19</t>
+          <t>2026/10/22</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026/10/28</t>
+          <t>2026/10/31</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/19~2026/10/28 (測試)</t>
+          <t>服務期間:2026/10/22~2026/10/31 (測試)</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026/06/03 17:56:03</t>
+          <t>2026/06/06 22:25:02</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1496,12 +1496,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026/08/30</t>
+          <t>2026/09/02</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026/09/03</t>
+          <t>2026/09/06</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/30~2026/09/03 (測試)</t>
+          <t>服務期間:2026/09/02~2026/09/06 (測試)</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026/07/14 12:53:44</t>
+          <t>2026/07/17 17:22:43</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026/11/21</t>
+          <t>2026/11/24</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026/11/29</t>
+          <t>2026/12/02</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/21~2026/11/29 (測試)</t>
+          <t>服務期間:2026/11/24~2026/12/02 (測試)</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026/07/01 17:11:15</t>
+          <t>2026/07/04 21:40:14</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1718,12 +1718,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026/11/23</t>
+          <t>2026/11/26</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026/11/30</t>
+          <t>2026/12/03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/23~2026/11/30 (測試)</t>
+          <t>服務期間:2026/11/26~2026/12/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026/06/01 19:42:33</t>
+          <t>2026/06/05 00:11:32</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1829,12 +1829,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026/09/20</t>
+          <t>2026/09/23</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/10~2026/09/20 (測試)</t>
+          <t>服務期間:2026/09/13~2026/09/23 (測試)</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026/06/07 17:20:42</t>
+          <t>2026/06/10 21:49:41</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026/11/11</t>
+          <t>2026/11/14</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026/11/16</t>
+          <t>2026/11/19</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/11~2026/11/16 (測試)</t>
+          <t>服務期間:2026/11/14~2026/11/19 (測試)</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026/05/31 02:20:38</t>
+          <t>2026/06/03 06:49:37</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2055,12 +2055,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026/08/29</t>
+          <t>2026/09/01</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026/09/05</t>
+          <t>2026/09/08</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/29~2026/09/05 (測試)</t>
+          <t>服務期間:2026/09/01~2026/09/08 (測試)</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026/05/30 21:41:47</t>
+          <t>2026/06/03 02:10:46</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2166,12 +2166,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026/11/10</t>
+          <t>2026/11/13</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026/11/19</t>
+          <t>2026/11/22</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/10~2026/11/19 (測試)</t>
+          <t>服務期間:2026/11/13~2026/11/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026/06/04 10:33:25</t>
+          <t>2026/06/07 15:02:24</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2277,12 +2277,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026/11/16</t>
+          <t>2026/11/19</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026/11/19</t>
+          <t>2026/11/22</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/16~2026/11/19 (測試)</t>
+          <t>服務期間:2026/11/19~2026/11/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026/06/23 16:24:49</t>
+          <t>2026/06/26 20:53:48</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2392,12 +2392,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026/09/02</t>
+          <t>2026/09/05</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/02~2026/09/10 (測試)</t>
+          <t>服務期間:2026/09/05~2026/09/13 (測試)</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026/07/11 07:59:40</t>
+          <t>2026/07/14 12:28:39</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026/11/28</t>
+          <t>2026/12/01</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026/12/04</t>
+          <t>2026/12/07</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/28~2026/12/04 (測試)</t>
+          <t>服務期間:2026/12/01~2026/12/07 (測試)</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026/06/25 21:07:42</t>
+          <t>2026/06/29 01:36:41</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2618,12 +2618,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026/10/06</t>
+          <t>2026/10/09</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026/10/12</t>
+          <t>2026/10/15</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/06~2026/10/12 (測試)</t>
+          <t>服務期間:2026/10/09~2026/10/15 (測試)</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026/07/03 12:42:34</t>
+          <t>2026/07/06 17:11:33</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2729,12 +2729,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026/10/24</t>
+          <t>2026/10/27</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026/10/31</t>
+          <t>2026/11/03</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/24~2026/10/31 (測試)</t>
+          <t>服務期間:2026/10/27~2026/11/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026/05/18 15:42:30</t>
+          <t>2026/05/21 20:11:29</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2027/01/07</t>
+          <t>2027/01/10</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2027/01/13</t>
+          <t>2027/01/16</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>服務期間:2027/01/07~2027/01/13 (測試)</t>
+          <t>服務期間:2027/01/10~2027/01/16 (測試)</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026/05/22 03:51:56</t>
+          <t>2026/05/25 08:20:55</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2955,12 +2955,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026/10/06</t>
+          <t>2026/10/09</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/06~2026/10/09 (測試)</t>
+          <t>服務期間:2026/10/09~2026/10/12 (測試)</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026/06/27 16:14:57</t>
+          <t>2026/06/30 20:43:56</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026/09/02</t>
+          <t>2026/09/05</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/02~2026/09/10 (測試)</t>
+          <t>服務期間:2026/09/05~2026/09/13 (測試)</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026/07/01 05:17:09</t>
+          <t>2026/07/04 09:46:08</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3177,12 +3177,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026/12/23</t>
+          <t>2026/12/26</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/23~2026/12/29 (測試)</t>
+          <t>服務期間:2026/12/26~2027/01/01 (測試)</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026/06/18 03:29:32</t>
+          <t>2026/06/21 07:58:31</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3288,12 +3288,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026/10/23</t>
+          <t>2026/10/26</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026/10/31</t>
+          <t>2026/11/03</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/23~2026/10/31 (測試)</t>
+          <t>服務期間:2026/10/26~2026/11/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026/07/02 18:04:07</t>
+          <t>2026/07/05 22:33:06</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3399,12 +3399,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026/11/08</t>
+          <t>2026/11/11</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026/11/18</t>
+          <t>2026/11/21</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/08~2026/11/18 (測試)</t>
+          <t>服務期間:2026/11/11~2026/11/21 (測試)</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3469,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026/07/12 05:20:54</t>
+          <t>2026/07/15 09:49:53</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3514,12 +3514,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026/12/19</t>
+          <t>2026/12/22</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/19~2026/12/29 (測試)</t>
+          <t>服務期間:2026/12/22~2027/01/01 (測試)</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026/06/02 23:50:03</t>
+          <t>2026/06/06 04:19:02</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026/08/24</t>
+          <t>2026/08/27</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/18~2026/08/24 (測試)</t>
+          <t>服務期間:2026/08/21~2026/08/27 (測試)</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026/07/09 02:48:57</t>
+          <t>2026/07/12 07:17:56</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3740,12 +3740,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026/10/15</t>
+          <t>2026/10/18</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026/10/25</t>
+          <t>2026/10/28</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/15~2026/10/25 (測試)</t>
+          <t>服務期間:2026/10/18~2026/10/28 (測試)</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026/05/30 05:07:50</t>
+          <t>2026/06/02 09:36:49</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3851,12 +3851,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026/12/15</t>
+          <t>2026/12/18</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026/12/21</t>
+          <t>2026/12/24</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/15~2026/12/21 (測試)</t>
+          <t>服務期間:2026/12/18~2026/12/24 (測試)</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026/07/02 18:25:54</t>
+          <t>2026/07/05 22:54:53</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3962,12 +3962,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026/11/25</t>
+          <t>2026/11/28</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026/12/04</t>
+          <t>2026/12/07</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/25~2026/12/04 (測試)</t>
+          <t>服務期間:2026/11/28~2026/12/07 (測試)</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026/07/01 04:18:24</t>
+          <t>2026/07/04 08:47:23</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4073,12 +4073,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026/11/25</t>
+          <t>2026/11/28</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026/12/02</t>
+          <t>2026/12/05</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/25~2026/12/02 (測試)</t>
+          <t>服務期間:2026/11/28~2026/12/05 (測試)</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026/06/17 02:22:18</t>
+          <t>2026/06/20 06:51:17</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4184,12 +4184,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026/12/27</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/27~2026/12/31 (測試)</t>
+          <t>服務期間:2026/12/30~2027/01/03 (測試)</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026/05/19 12:00:38</t>
+          <t>2026/05/22 16:29:37</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026/09/07</t>
+          <t>2026/09/10</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026/09/12</t>
+          <t>2026/09/15</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/07~2026/09/12 (測試)</t>
+          <t>服務期間:2026/09/10~2026/09/15 (測試)</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026/05/20 04:02:51</t>
+          <t>2026/05/23 08:31:50</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4406,12 +4406,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026/10/05</t>
+          <t>2026/10/08</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/05~2026/10/09 (測試)</t>
+          <t>服務期間:2026/10/08~2026/10/12 (測試)</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026/06/25 22:27:49</t>
+          <t>2026/06/29 02:56:49</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4517,12 +4517,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026/11/08</t>
+          <t>2026/11/11</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026/11/15</t>
+          <t>2026/11/18</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>服務期間:2026/11/08~2026/11/15 (測試)</t>
+          <t>服務期間:2026/11/11~2026/11/18 (測試)</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026/06/03 19:55:54</t>
+          <t>2026/06/07 00:24:54</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4628,12 +4628,12 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026/10/22</t>
+          <t>2026/10/25</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026/10/26</t>
+          <t>2026/10/29</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/22~2026/10/26 (測試)</t>
+          <t>服務期間:2026/10/25~2026/10/29 (測試)</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026/05/27 13:18:06</t>
+          <t>2026/05/30 17:47:06</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4739,12 +4739,12 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026/10/17</t>
+          <t>2026/10/20</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/09~2026/10/17 (測試)</t>
+          <t>服務期間:2026/10/12~2026/10/20 (測試)</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026/06/06 13:40:45</t>
+          <t>2026/06/09 18:09:45</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4850,12 +4850,12 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026/10/30</t>
+          <t>2026/11/02</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026/11/04</t>
+          <t>2026/11/07</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/30~2026/11/04 (測試)</t>
+          <t>服務期間:2026/11/02~2026/11/07 (測試)</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026/07/04 22:57:15</t>
+          <t>2026/07/08 03:26:15</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026/09/13</t>
+          <t>2026/09/16</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026/09/20</t>
+          <t>2026/09/23</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/13~2026/09/20 (測試)</t>
+          <t>服務期間:2026/09/16~2026/09/23 (測試)</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026/05/18 12:14:34</t>
+          <t>2026/05/21 16:43:34</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5072,12 +5072,12 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026/09/04</t>
+          <t>2026/09/07</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026/09/08</t>
+          <t>2026/09/11</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/04~2026/09/08 (測試)</t>
+          <t>服務期間:2026/09/07~2026/09/11 (測試)</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026/07/02 18:00:39</t>
+          <t>2026/07/05 22:29:39</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5183,12 +5183,12 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026/09/10</t>
+          <t>2026/09/13</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026/09/16</t>
+          <t>2026/09/19</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/10~2026/09/16 (測試)</t>
+          <t>服務期間:2026/09/13~2026/09/19 (測試)</t>
         </is>
       </c>
     </row>
@@ -5249,7 +5249,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026/06/03 08:39:08</t>
+          <t>2026/06/06 13:08:08</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5294,12 +5294,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026/09/29</t>
+          <t>2026/10/02</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026/10/09</t>
+          <t>2026/10/12</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>服務期間:2026/09/29~2026/10/09 (測試)</t>
+          <t>服務期間:2026/10/02~2026/10/12 (測試)</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026/06/17 20:45:08</t>
+          <t>2026/06/21 01:14:08</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5409,12 +5409,12 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2026/08/30</t>
+          <t>2026/09/02</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026/09/05</t>
+          <t>2026/09/08</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/30~2026/09/05 (測試)</t>
+          <t>服務期間:2026/09/02~2026/09/08 (測試)</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026/06/26 09:10:45</t>
+          <t>2026/06/29 13:39:45</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5520,12 +5520,12 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2026/08/18</t>
+          <t>2026/08/21</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026/08/25</t>
+          <t>2026/08/28</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/18~2026/08/25 (測試)</t>
+          <t>服務期間:2026/08/21~2026/08/28 (測試)</t>
         </is>
       </c>
     </row>
@@ -5586,7 +5586,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026/06/26 16:01:29</t>
+          <t>2026/06/29 20:30:29</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5631,12 +5631,12 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026/12/03</t>
+          <t>2026/12/06</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026/12/08</t>
+          <t>2026/12/11</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>服務期間:2026/12/03~2026/12/08 (測試)</t>
+          <t>服務期間:2026/12/06~2026/12/11 (測試)</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026/05/25 05:11:52</t>
+          <t>2026/05/28 09:40:52</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5742,12 +5742,12 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2027/01/10</t>
+          <t>2027/01/13</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2027/01/19</t>
+          <t>2027/01/22</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5789,7 +5789,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>服務期間:2027/01/10~2027/01/19 (測試)</t>
+          <t>服務期間:2027/01/13~2027/01/22 (測試)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026/05/29 16:53:54</t>
+          <t>2026/06/01 21:22:54</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5853,12 +5853,12 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026/10/14</t>
+          <t>2026/10/17</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026/10/23</t>
+          <t>2026/10/26</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/14~2026/10/23 (測試)</t>
+          <t>服務期間:2026/10/17~2026/10/26 (測試)</t>
         </is>
       </c>
     </row>
@@ -5923,7 +5923,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026/06/04 21:10:58</t>
+          <t>2026/06/08 01:39:58</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5968,12 +5968,12 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026/08/16</t>
+          <t>2026/08/19</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026/08/26</t>
+          <t>2026/08/29</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>服務期間:2026/08/16~2026/08/26 (測試)</t>
+          <t>服務期間:2026/08/19~2026/08/29 (測試)</t>
         </is>
       </c>
     </row>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026/06/17 06:48:49</t>
+          <t>2026/06/20 11:17:49</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -6083,12 +6083,12 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026/10/22</t>
+          <t>2026/10/25</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026/10/27</t>
+          <t>2026/10/30</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>服務期間:2026/10/22~2026/10/27 (測試)</t>
+          <t>服務期間:2026/10/25~2026/10/30 (測試)</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026/05/19 15:35:47</t>
+          <t>2026/05/22 20:04:47</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026/06/20 10:24:02</t>
+          <t>2026/06/23 14:53:02</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026/06/29 14:36:34</t>
+          <t>2026/07/02 19:05:34</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026/06/06 16:36:08</t>
+          <t>2026/06/09 21:05:08</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -7304,7 +7304,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026/05/16 03:56:18</t>
+          <t>2026/05/19 08:25:18</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026/05/23 13:32:37</t>
+          <t>2026/05/26 18:01:37</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026/05/19 00:32:03</t>
+          <t>2026/05/22 05:01:03</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026/05/26 09:37:08</t>
+          <t>2026/05/29 14:06:08</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -8172,7 +8172,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026/06/18 18:50:29</t>
+          <t>2026/06/21 23:19:29</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026/06/12 04:43:00</t>
+          <t>2026/06/15 09:12:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026/06/21 14:01:34</t>
+          <t>2026/06/24 18:30:34</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026/06/20 20:27:40</t>
+          <t>2026/06/24 00:56:40</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026/05/29 11:28:31</t>
+          <t>2026/06/01 15:57:31</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -9261,7 +9261,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026/05/15 11:13:18</t>
+          <t>2026/05/18 15:42:18</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026/05/16 12:08:14</t>
+          <t>2026/05/19 16:37:14</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026/06/20 15:47:45</t>
+          <t>2026/06/23 20:16:45</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026/06/28 03:24:22</t>
+          <t>2026/07/01 07:53:22</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -10157,7 +10157,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026/06/15 06:42:21</t>
+          <t>2026/06/18 11:11:21</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -10378,7 +10378,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026/05/17 20:29:55</t>
+          <t>2026/05/21 00:58:55</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -10599,7 +10599,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026/06/13 07:59:22</t>
+          <t>2026/06/16 12:28:22</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026/06/19 12:52:40</t>
+          <t>2026/06/22 17:21:40</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026/05/23 06:04:12</t>
+          <t>2026/05/26 10:33:12</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -11282,7 +11282,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026/07/08 04:19:46</t>
+          <t>2026/07/11 08:48:46</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -11495,7 +11495,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026/07/03 07:26:50</t>
+          <t>2026/07/06 11:55:50</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026/05/28 12:24:00</t>
+          <t>2026/05/31 16:53:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026/06/14 08:12:22</t>
+          <t>2026/06/17 12:41:22</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026/05/24 10:46:53</t>
+          <t>2026/05/27 15:15:53</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -12391,7 +12391,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026/06/10 06:27:54</t>
+          <t>2026/06/13 10:56:54</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -12620,7 +12620,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026/05/18 00:25:35</t>
+          <t>2026/05/21 04:54:35</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -12837,7 +12837,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026/06/19 08:39:46</t>
+          <t>2026/06/22 13:08:46</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026/07/01 00:39:29</t>
+          <t>2026/07/04 05:08:29</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026/06/29 13:12:13</t>
+          <t>2026/07/02 17:41:13</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026/05/18 00:53:02</t>
+          <t>2026/05/21 05:22:02</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026/07/01 21:19:08</t>
+          <t>2026/07/05 01:48:08</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -13946,7 +13946,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026/05/23 03:11:48</t>
+          <t>2026/05/26 07:40:48</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -14159,7 +14159,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026/06/15 03:09:33</t>
+          <t>2026/06/18 07:38:33</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026/07/12 09:06:12</t>
+          <t>2026/07/15 13:35:12</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -14593,7 +14593,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026/05/15 14:48:53</t>
+          <t>2026/05/18 19:17:53</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -14818,7 +14818,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026/05/24 02:36:03</t>
+          <t>2026/05/27 07:05:03</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -15047,7 +15047,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026/06/06 11:18:19</t>
+          <t>2026/06/09 15:47:19</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -15268,7 +15268,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026/07/07 07:17:01</t>
+          <t>2026/07/10 11:46:01</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026/07/05 03:54:24</t>
+          <t>2026/07/08 08:23:24</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -15730,7 +15730,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026/07/07 00:51:56</t>
+          <t>2026/07/10 05:20:56</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -15939,7 +15939,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026/06/26 20:54:42</t>
+          <t>2026/06/30 01:23:42</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -16152,7 +16152,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026/05/18 01:40:47</t>
+          <t>2026/05/21 06:09:47</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -16369,7 +16369,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026/06/23 18:58:40</t>
+          <t>2026/06/26 23:27:40</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -16590,7 +16590,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026/07/08 14:56:16</t>
+          <t>2026/07/11 19:25:16</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026/07/04 07:51:15</t>
+          <t>2026/07/07 12:20:15</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -17000,7 +17000,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026/05/17 20:06:39</t>
+          <t>2026/05/21 00:35:39</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -17217,7 +17217,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026/07/03 08:08:29</t>
+          <t>2026/07/06 12:37:29</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -17920,7 +17920,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>06-15 07:17</t>
+          <t>06-18 11:46</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -18224,7 +18224,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>06-03 23:04</t>
+          <t>06-07 03:33</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -18520,7 +18520,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>06-20 05:41</t>
+          <t>06-23 10:10</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -18820,7 +18820,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>07-05 19:00</t>
+          <t>07-08 23:29</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -19120,7 +19120,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>06-24 19:41</t>
+          <t>06-28 00:10</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -19416,7 +19416,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>06-07 18:44</t>
+          <t>06-10 23:13</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -19736,7 +19736,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>06-04 07:50</t>
+          <t>06-07 12:19</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -20036,7 +20036,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>07-04 19:17</t>
+          <t>07-07 23:46</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -20344,7 +20344,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>06-03 17:56</t>
+          <t>06-06 22:25</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -20644,7 +20644,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>07-14 12:53</t>
+          <t>07-17 17:22</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -20956,7 +20956,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>07-01 17:11</t>
+          <t>07-04 21:40</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -21252,7 +21252,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>06-01 19:42</t>
+          <t>06-05 00:11</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -21552,7 +21552,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>06-07 17:20</t>
+          <t>06-10 21:49</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -21852,7 +21852,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>05-31 02:20</t>
+          <t>06-03 06:49</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -22168,7 +22168,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>05-30 21:41</t>
+          <t>06-03 02:10</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -22496,7 +22496,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>06-04 10:33</t>
+          <t>06-07 15:02</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -22788,7 +22788,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>06-23 16:24</t>
+          <t>06-26 20:53</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -23072,7 +23072,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>07-11 07:59</t>
+          <t>07-14 12:28</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -23380,7 +23380,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>06-25 21:07</t>
+          <t>06-29 01:36</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -23680,7 +23680,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>07-03 12:42</t>
+          <t>07-06 17:11</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -23988,7 +23988,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>05-18 15:42</t>
+          <t>05-21 20:11</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -24268,7 +24268,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>05-22 03:51</t>
+          <t>05-25 08:20</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -24572,7 +24572,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>06-27 16:14</t>
+          <t>06-30 20:43</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -24884,7 +24884,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>07-01 05:17</t>
+          <t>07-04 09:46</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>06-18 03:29</t>
+          <t>06-21 07:58</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -25500,7 +25500,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>07-02 18:04</t>
+          <t>07-05 22:33</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -25800,7 +25800,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>07-12 05:20</t>
+          <t>07-15 09:49</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -26100,7 +26100,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>06-02 23:50</t>
+          <t>06-06 04:19</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -26408,7 +26408,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>07-09 02:48</t>
+          <t>07-12 07:17</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -26720,7 +26720,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>05-30 05:07</t>
+          <t>06-02 09:36</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -27008,7 +27008,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>07-02 18:25</t>
+          <t>07-05 22:54</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -27304,7 +27304,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>07-01 04:18</t>
+          <t>07-04 08:47</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -27604,7 +27604,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>06-17 02:22</t>
+          <t>06-20 06:51</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -27892,7 +27892,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>05-19 12:00</t>
+          <t>05-22 16:29</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -28204,7 +28204,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>05-20 04:02</t>
+          <t>05-23 08:31</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -28516,7 +28516,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>06-25 22:27</t>
+          <t>06-29 02:56</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -28808,7 +28808,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>06-03 19:55</t>
+          <t>06-07 00:24</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -29092,7 +29092,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>05-27 13:18</t>
+          <t>05-30 17:47</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -29404,7 +29404,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>06-06 13:40</t>
+          <t>06-09 18:09</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -29708,7 +29708,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>07-04 22:57</t>
+          <t>07-08 03:26</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -30000,7 +30000,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>05-18 12:14</t>
+          <t>05-21 16:43</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -30304,7 +30304,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>07-02 18:00</t>
+          <t>07-05 22:29</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -30600,7 +30600,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>06-03 08:39</t>
+          <t>06-06 13:08</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -30920,7 +30920,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>06-17 20:45</t>
+          <t>06-21 01:14</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -31228,7 +31228,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>06-26 09:10</t>
+          <t>06-29 13:39</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -31536,7 +31536,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>06-26 16:01</t>
+          <t>06-29 20:30</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -31844,7 +31844,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>05-25 05:11</t>
+          <t>05-28 09:40</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -32132,7 +32132,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>05-29 16:53</t>
+          <t>06-01 21:22</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -32428,7 +32428,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>06-04 21:10</t>
+          <t>06-08 01:39</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -32728,7 +32728,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>06-17 06:48</t>
+          <t>06-20 11:17</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">

</xml_diff>